<commit_message>
version stable fiche de prime  module PRIME
</commit_message>
<xml_diff>
--- a/docs/samples/EXEMPLAIRE PRIME1.xlsx
+++ b/docs/samples/EXEMPLAIRE PRIME1.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="38">
   <si>
     <t>Répartitions des RDV</t>
   </si>
@@ -138,30 +138,6 @@
   </si>
   <si>
     <t>Somme SAV</t>
-  </si>
-  <si>
-    <t>Plafond Prime</t>
-  </si>
-  <si>
-    <t>Plafond Challenge</t>
-  </si>
-  <si>
-    <t>Cellule</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PEC callback client </t>
-  </si>
-  <si>
-    <t>Taux de tickets affectés en - de 6h ouvrées IND  de groupe</t>
-  </si>
-  <si>
-    <t>Qualite de traitement (picking 20 dossier)</t>
-  </si>
-  <si>
-    <t>Somme Indicateurs Cellules</t>
-  </si>
-  <si>
-    <t>TOTAL Général</t>
   </si>
 </sst>
 </file>
@@ -172,7 +148,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.00\ _€"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -292,58 +268,8 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
-      <sz val="10"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="22">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -420,55 +346,8 @@
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6ECD1"/>
-        <bgColor rgb="FFC6ECD1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFECF4FA"/>
-        <bgColor rgb="FFECF4FA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFDFF5E5"/>
-        <bgColor rgb="FFDFF5E5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC5E0B3"/>
-        <bgColor rgb="FFC5E0B3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF0070C0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="37">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -664,263 +543,16 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="7">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="14" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1132,119 +764,8 @@
     <xf numFmtId="10" fontId="10" fillId="0" borderId="10" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="16" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="20" fillId="17" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="11" fillId="18" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="20" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="12" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="20" fillId="19" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="20" fillId="17" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="11" fillId="18" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="20" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="12" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="20" fillId="19" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="11" fillId="18" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="20" fillId="19" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="22" fillId="20" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="20" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="20" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="23" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="23" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="23" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="7">
-    <cellStyle name="Calcul" xfId="6" builtinId="22"/>
+  <cellStyles count="6">
     <cellStyle name="Neutre 2" xfId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="4"/>
@@ -1589,14 +1110,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R37"/>
+  <dimension ref="A1:P37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32.5546875" customWidth="1"/>
     <col min="17" max="17" width="18.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="57"/>
       <c r="B1" s="57"/>
       <c r="C1" s="57"/>
@@ -1619,14 +1140,8 @@
       <c r="N1" s="60"/>
       <c r="O1" s="60"/>
       <c r="P1" s="60"/>
-      <c r="Q1" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" ht="107.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:16" ht="107.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="61" t="s">
         <v>3</v>
       </c>
@@ -1667,14 +1182,8 @@
       <c r="P2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="Q2" s="71">
-        <v>1000</v>
-      </c>
-      <c r="R2" s="71">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6"/>
       <c r="B3" s="62" t="s">
         <v>11</v>
@@ -1721,10 +1230,8 @@
         <f>IF(ISBLANK(L3),"",(N3*#REF!)*O3)</f>
         <v/>
       </c>
-      <c r="Q3" s="72"/>
-      <c r="R3" s="72"/>
-    </row>
-    <row r="4" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="6"/>
       <c r="B4" s="64"/>
       <c r="C4" s="65"/>
@@ -1757,10 +1264,8 @@
       <c r="N4" s="15"/>
       <c r="O4" s="11"/>
       <c r="P4" s="12"/>
-      <c r="Q4" s="73"/>
-      <c r="R4" s="73"/>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" s="16"/>
       <c r="B5" s="66"/>
       <c r="C5" s="67"/>
@@ -1793,10 +1298,8 @@
       <c r="N5" s="15"/>
       <c r="O5" s="11"/>
       <c r="P5" s="12"/>
-      <c r="Q5" s="73"/>
-      <c r="R5" s="73"/>
-    </row>
-    <row r="6" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="16"/>
       <c r="B6" s="42" t="s">
         <v>15</v>
@@ -1822,7 +1325,7 @@
       </c>
       <c r="K6" s="12">
         <f>IF(ISBLANK(F6),"",(I6*Q2)*J6)</f>
-        <v>67.34000000000006</v>
+        <v>0</v>
       </c>
       <c r="L6" s="13"/>
       <c r="M6" s="14">
@@ -1839,10 +1342,8 @@
         <f>IF(ISBLANK(L6),"",(N6*#REF!)*O6)</f>
         <v/>
       </c>
-      <c r="Q6" s="73"/>
-      <c r="R6" s="73"/>
-    </row>
-    <row r="7" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="6"/>
       <c r="B7" s="42" t="s">
         <v>16</v>
@@ -1868,7 +1369,7 @@
       </c>
       <c r="K7" s="12">
         <f>IF(ISBLANK(F7),"",(I7*Q2)*J7)</f>
-        <v>1.5299999999999965</v>
+        <v>0</v>
       </c>
       <c r="L7" s="9"/>
       <c r="M7" s="10">
@@ -1885,10 +1386,8 @@
         <f>IF(ISBLANK(L7),"",(N7*#REF!)*O7)</f>
         <v/>
       </c>
-      <c r="Q7" s="73"/>
-      <c r="R7" s="73"/>
-    </row>
-    <row r="8" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6"/>
       <c r="B8" s="42" t="s">
         <v>17</v>
@@ -1914,7 +1413,7 @@
       </c>
       <c r="K8" s="12">
         <f>IF(ISBLANK(F8),"",(I8*Q2)*J8)</f>
-        <v>17.189999999999998</v>
+        <v>0</v>
       </c>
       <c r="L8" s="9"/>
       <c r="M8" s="10">
@@ -1931,10 +1430,8 @@
         <f>IF(ISBLANK(L8),"",(N8*#REF!)*O8)</f>
         <v/>
       </c>
-      <c r="Q8" s="73"/>
-      <c r="R8" s="73"/>
-    </row>
-    <row r="9" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="6"/>
       <c r="B9" s="42" t="s">
         <v>18</v>
@@ -1977,10 +1474,8 @@
         <f>IF(ISBLANK(L9),"",(N9*#REF!)*O9)</f>
         <v/>
       </c>
-      <c r="Q9" s="73"/>
-      <c r="R9" s="73"/>
-    </row>
-    <row r="10" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="6"/>
       <c r="B10" s="42" t="s">
         <v>19</v>
@@ -2012,7 +1507,7 @@
       </c>
       <c r="K10" s="47">
         <f>IF(ISBLANK(F10),"",(I10*Q2)*((J10+J11+J12+J13+J14+J15+J16+J17+J18)))</f>
-        <v>60.671267554112596</v>
+        <v>0</v>
       </c>
       <c r="L10" s="13"/>
       <c r="M10" s="14">
@@ -2029,10 +1524,8 @@
         <f>IF(ISBLANK(L10),"",(N10*R2)*((O18+O10+O11+O12+O13+O14+O15+O16+O17)))</f>
         <v/>
       </c>
-      <c r="Q10" s="73"/>
-      <c r="R10" s="73"/>
-    </row>
-    <row r="11" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>22</v>
       </c>
@@ -2069,10 +1562,8 @@
         <v/>
       </c>
       <c r="P11" s="54"/>
-      <c r="Q11" s="73"/>
-      <c r="R11" s="73"/>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
       <c r="B12" s="42"/>
       <c r="C12" s="42"/>
@@ -2107,10 +1598,8 @@
         <v/>
       </c>
       <c r="P12" s="54"/>
-      <c r="Q12" s="73"/>
-      <c r="R12" s="73"/>
-    </row>
-    <row r="13" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="6"/>
       <c r="B13" s="42"/>
       <c r="C13" s="42" t="s">
@@ -2147,10 +1636,8 @@
         <v/>
       </c>
       <c r="P13" s="54"/>
-      <c r="Q13" s="73"/>
-      <c r="R13" s="73"/>
-    </row>
-    <row r="14" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="6"/>
       <c r="B14" s="42"/>
       <c r="C14" s="42"/>
@@ -2185,10 +1672,8 @@
         <v/>
       </c>
       <c r="P14" s="54"/>
-      <c r="Q14" s="73"/>
-      <c r="R14" s="73"/>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" s="6"/>
       <c r="B15" s="42"/>
       <c r="C15" s="42"/>
@@ -2223,10 +1708,8 @@
         <v/>
       </c>
       <c r="P15" s="54"/>
-      <c r="Q15" s="73"/>
-      <c r="R15" s="73"/>
-    </row>
-    <row r="16" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="6"/>
       <c r="B16" s="42"/>
       <c r="C16" s="42" t="s">
@@ -2263,10 +1746,8 @@
         <v/>
       </c>
       <c r="P16" s="54"/>
-      <c r="Q16" s="73"/>
-      <c r="R16" s="73"/>
-    </row>
-    <row r="17" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="6"/>
       <c r="B17" s="42"/>
       <c r="C17" s="42"/>
@@ -2301,10 +1782,8 @@
         <v/>
       </c>
       <c r="P17" s="54"/>
-      <c r="Q17" s="73"/>
-      <c r="R17" s="73"/>
-    </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A18" s="6"/>
       <c r="B18" s="42"/>
       <c r="C18" s="42"/>
@@ -2339,10 +1818,8 @@
         <v/>
       </c>
       <c r="P18" s="55"/>
-      <c r="Q18" s="73"/>
-      <c r="R18" s="73"/>
-    </row>
-    <row r="19" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="6"/>
       <c r="B19" s="42" t="s">
         <v>27</v>
@@ -2372,7 +1849,7 @@
       </c>
       <c r="K19" s="47">
         <f>IF(ISBLANK(F19),"",(I19*Q2)*(J19+J20+J21))</f>
-        <v>68.723853333333352</v>
+        <v>0</v>
       </c>
       <c r="L19" s="13"/>
       <c r="M19" s="14">
@@ -2389,10 +1866,8 @@
         <f>IF(ISBLANK(L19),"",(N19*#REF!)*(O19+O20+O21))</f>
         <v/>
       </c>
-      <c r="Q19" s="73"/>
-      <c r="R19" s="73"/>
-    </row>
-    <row r="20" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="6"/>
       <c r="B20" s="42"/>
       <c r="C20" s="43" t="s">
@@ -2427,10 +1902,8 @@
         <v/>
       </c>
       <c r="P20" s="48"/>
-      <c r="Q20" s="73"/>
-      <c r="R20" s="73"/>
-    </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
       <c r="B21" s="42"/>
       <c r="C21" s="43" t="s">
@@ -2465,10 +1938,8 @@
         <v/>
       </c>
       <c r="P21" s="49"/>
-      <c r="Q21" s="73"/>
-      <c r="R21" s="73"/>
-    </row>
-    <row r="22" spans="1:18" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A22" s="6"/>
       <c r="B22" s="37" t="s">
         <v>28</v>
@@ -2486,7 +1957,7 @@
       <c r="J22" s="23"/>
       <c r="K22" s="24">
         <f>SUM(K6:K21)</f>
-        <v>215.45512088744601</v>
+        <v>0</v>
       </c>
       <c r="L22" s="37"/>
       <c r="M22" s="37"/>
@@ -2499,10 +1970,8 @@
         <f>SUM(P6:P20)</f>
         <v>0</v>
       </c>
-      <c r="Q22" s="73"/>
-      <c r="R22" s="73"/>
-    </row>
-    <row r="23" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="38" t="s">
         <v>29</v>
       </c>
@@ -2545,10 +2014,8 @@
         <f>IF(ISBLANK(L23),"",(N23*#REF!)*O23)</f>
         <v/>
       </c>
-      <c r="Q23" s="73"/>
-      <c r="R23" s="73"/>
-    </row>
-    <row r="24" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="38"/>
       <c r="B24" s="39" t="s">
         <v>31</v>
@@ -2589,10 +2056,8 @@
         <f>IF(ISBLANK(L24),"",(N24*#REF!)*O24)</f>
         <v/>
       </c>
-      <c r="Q24" s="73"/>
-      <c r="R24" s="73"/>
-    </row>
-    <row r="25" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="38"/>
       <c r="B25" s="39" t="s">
         <v>32</v>
@@ -2633,10 +2098,8 @@
         <f>IF(ISBLANK(L25),"",(N25*#REF!)*O25)</f>
         <v/>
       </c>
-      <c r="Q25" s="73"/>
-      <c r="R25" s="73"/>
-    </row>
-    <row r="26" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="26" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="38"/>
       <c r="B26" s="39" t="s">
         <v>33</v>
@@ -2677,10 +2140,8 @@
         <f>IF(ISBLANK(L26),"",(N26*#REF!)*O26)</f>
         <v/>
       </c>
-      <c r="Q26" s="73"/>
-      <c r="R26" s="73"/>
-    </row>
-    <row r="27" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="27" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="38"/>
       <c r="B27" s="39" t="s">
         <v>34</v>
@@ -2721,10 +2182,8 @@
         <f>IF(ISBLANK(L27),"",(N27*#REF!)*O27)</f>
         <v/>
       </c>
-      <c r="Q27" s="73"/>
-      <c r="R27" s="73"/>
-    </row>
-    <row r="28" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="28" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="38"/>
       <c r="B28" s="39" t="s">
         <v>35</v>
@@ -2765,10 +2224,8 @@
         <f>IF(ISBLANK(L28),"",(N28*#REF!)*O28)</f>
         <v/>
       </c>
-      <c r="Q28" s="73"/>
-      <c r="R28" s="73"/>
-    </row>
-    <row r="29" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="29" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="38"/>
       <c r="B29" s="39" t="s">
         <v>36</v>
@@ -2809,10 +2266,8 @@
         <f>IF(ISBLANK(L29),"",(N29*#REF!)*O29)</f>
         <v/>
       </c>
-      <c r="Q29" s="73"/>
-      <c r="R29" s="73"/>
-    </row>
-    <row r="30" spans="1:18" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="30" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="38"/>
       <c r="B30" s="37" t="s">
         <v>37</v>
@@ -2843,229 +2298,16 @@
         <f>SUM(P23:P29)</f>
         <v>0</v>
       </c>
-      <c r="Q30" s="73"/>
-      <c r="R30" s="73"/>
-    </row>
-    <row r="31" spans="1:18" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="74" t="s">
-        <v>40</v>
-      </c>
-      <c r="B31" s="75" t="s">
-        <v>41</v>
-      </c>
-      <c r="C31" s="76"/>
-      <c r="D31" s="77"/>
-      <c r="E31" s="78"/>
-      <c r="F31" s="79"/>
-      <c r="G31" s="80">
-        <v>0.9</v>
-      </c>
-      <c r="H31" s="80">
-        <v>1</v>
-      </c>
-      <c r="I31" s="81">
-        <v>0.2</v>
-      </c>
-      <c r="J31" s="82" t="str">
-        <f t="shared" ref="J31:J33" si="5">IF(ISBLANK(F31),"",IF(F31&lt;G31,0,IF(F31=G31,0.1,IF(F31&gt;=H31,1,((F31-G31)/(H31-G31))))))</f>
-        <v/>
-      </c>
-      <c r="K31" s="83" t="str">
-        <f>IF(ISBLANK(F31),"",(I31*Q2)*J31)</f>
-        <v/>
-      </c>
-      <c r="L31" s="84"/>
-      <c r="M31" s="80">
-        <v>0.4</v>
-      </c>
-      <c r="N31" s="81">
-        <v>0</v>
-      </c>
-      <c r="O31" s="82" t="str">
-        <f t="shared" ref="O31:O33" si="6">IF(ISBLANK(L31),"",IF(L31&lt;M31,0,IF(L31&gt;=M31,1)))</f>
-        <v/>
-      </c>
-      <c r="P31" s="83" t="str">
-        <f>IF(ISBLANK(L31),"",(N31*#REF!)*O31)</f>
-        <v/>
-      </c>
-      <c r="Q31" s="73"/>
-      <c r="R31" s="73"/>
-    </row>
-    <row r="32" spans="1:18" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="74"/>
-      <c r="B32" s="85" t="s">
-        <v>42</v>
-      </c>
-      <c r="C32" s="86"/>
-      <c r="D32" s="87"/>
-      <c r="E32" s="88"/>
-      <c r="F32" s="89"/>
-      <c r="G32" s="90">
-        <v>90</v>
-      </c>
-      <c r="H32" s="90">
-        <v>98</v>
-      </c>
-      <c r="I32" s="91">
-        <v>0.1</v>
-      </c>
-      <c r="J32" s="92" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="K32" s="83" t="str">
-        <f>IF(ISBLANK(F32),"",(I32*Q2)*J32)</f>
-        <v/>
-      </c>
-      <c r="L32" s="93"/>
-      <c r="M32" s="94">
-        <v>0.6</v>
-      </c>
-      <c r="N32" s="91">
-        <v>0</v>
-      </c>
-      <c r="O32" s="18" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="P32" s="95" t="str">
-        <f>IF(ISBLANK(L32),"",(N32*#REF!)*O32)</f>
-        <v/>
-      </c>
-      <c r="Q32" s="73"/>
-      <c r="R32" s="73"/>
-    </row>
-    <row r="33" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="74"/>
-      <c r="B33" s="85" t="s">
-        <v>43</v>
-      </c>
-      <c r="C33" s="86"/>
-      <c r="D33" s="87"/>
-      <c r="E33" s="96"/>
-      <c r="F33" s="89"/>
-      <c r="G33" s="90">
-        <v>17</v>
-      </c>
-      <c r="H33" s="90">
-        <v>20</v>
-      </c>
-      <c r="I33" s="91">
-        <v>0.2</v>
-      </c>
-      <c r="J33" s="92" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="K33" s="83" t="str">
-        <f>IF(ISBLANK(F33),"",(I33*Q2)*J33)</f>
-        <v/>
-      </c>
-      <c r="L33" s="97"/>
-      <c r="M33" s="90">
-        <v>10</v>
-      </c>
-      <c r="N33" s="91">
-        <v>0</v>
-      </c>
-      <c r="O33" s="18" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="P33" s="95" t="str">
-        <f>IF(ISBLANK(L33),"",(N33*#REF!)*O33)</f>
-        <v/>
-      </c>
-      <c r="Q33" s="73"/>
-      <c r="R33" s="73"/>
-    </row>
-    <row r="34" spans="1:18" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="74"/>
-      <c r="B34" s="98" t="s">
-        <v>44</v>
-      </c>
-      <c r="C34" s="99"/>
-      <c r="D34" s="99"/>
-      <c r="E34" s="99"/>
-      <c r="F34" s="99"/>
-      <c r="G34" s="99"/>
-      <c r="H34" s="100"/>
-      <c r="I34" s="101">
-        <f>SUM(I31:I33)</f>
-        <v>0.5</v>
-      </c>
-      <c r="J34" s="102"/>
-      <c r="K34" s="103">
-        <f>SUM(K31:K33)</f>
-        <v>0</v>
-      </c>
-      <c r="L34" s="104"/>
-      <c r="M34" s="105"/>
-      <c r="N34" s="101">
-        <f>SUM(N31:N33)</f>
-        <v>0</v>
-      </c>
-      <c r="O34" s="102"/>
-      <c r="P34" s="106">
-        <f>SUM(P31:P33)</f>
-        <v>0</v>
-      </c>
-      <c r="Q34" s="107"/>
-      <c r="R34" s="107"/>
-    </row>
-    <row r="35" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="108" t="s">
-        <v>45</v>
-      </c>
-      <c r="B35" s="108"/>
-      <c r="C35" s="108"/>
-      <c r="D35" s="108"/>
-      <c r="E35" s="108"/>
-      <c r="F35" s="108"/>
-      <c r="G35" s="108"/>
-      <c r="H35" s="108"/>
-      <c r="I35" s="109">
-        <f>I30+I22+I34</f>
-        <v>1</v>
-      </c>
-      <c r="J35" s="110"/>
-      <c r="K35" s="111">
-        <f>K30+K22+K34</f>
-        <v>215.45512088744601</v>
-      </c>
-      <c r="L35" s="108"/>
-      <c r="M35" s="108"/>
-      <c r="N35" s="109">
-        <f>N30+N22+N34</f>
-        <v>0.8</v>
-      </c>
-      <c r="O35" s="110"/>
-      <c r="P35" s="111">
-        <f>P30+P22+P34</f>
-        <v>0</v>
-      </c>
-      <c r="Q35" s="112">
-        <f>P35+K35</f>
-        <v>215.45512088744601</v>
-      </c>
-      <c r="R35" s="108"/>
-    </row>
-    <row r="36" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="37" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    </row>
+    <row r="31" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="32" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="33" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="34" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="35" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="36" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="37" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <mergeCells count="51">
-    <mergeCell ref="Q3:Q34"/>
-    <mergeCell ref="R3:R34"/>
-    <mergeCell ref="A31:A34"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="E31:E33"/>
-    <mergeCell ref="B34:H34"/>
-    <mergeCell ref="A35:H35"/>
-    <mergeCell ref="L35:M35"/>
-    <mergeCell ref="Q35:R35"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="B33:D33"/>
+  <mergeCells count="40">
     <mergeCell ref="L1:P1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="B3:C5"/>
@@ -3107,16 +2349,6 @@
     <mergeCell ref="B28:E28"/>
     <mergeCell ref="B29:E29"/>
   </mergeCells>
-  <conditionalFormatting sqref="I35">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
-      <formula>1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N35">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
-      <formula>1</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>